<commit_message>
feat: add centralized configuration and implement initial data exploration script
</commit_message>
<xml_diff>
--- a/output/QAQC_individus.xlsx
+++ b/output/QAQC_individus.xlsx
@@ -1,18 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resume" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Manquants" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Aberrants" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Distributions" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coherence" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Estimations" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Resume" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Manquants" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Aberrants" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Distributions" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Coherence" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Estimations" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -501,7 +501,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-06-27 23:57</t>
+          <t>2026-06-28 00:55</t>
         </is>
       </c>
     </row>
@@ -564,7 +564,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="9">
@@ -2652,7 +2652,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:D5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="19" customWidth="1" min="1" max="1"/>
@@ -2722,54 +2722,36 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>lien_cm_unique</t>
+          <t>sexe_manquant</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Plus d'un CM dans le menage</t>
+          <t>Sexe manquant</t>
         </is>
       </c>
       <c r="C4" s="3" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>sexe_manquant</t>
+          <t>age_manquant</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Sexe manquant</t>
+          <t>Age manquant</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>0</v>
+        <v>185</v>
       </c>
       <c r="D5" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="3" t="inlineStr">
-        <is>
-          <t>age_manquant</t>
-        </is>
-      </c>
-      <c r="B6" s="3" t="inlineStr">
-        <is>
-          <t>Age manquant</t>
-        </is>
-      </c>
-      <c r="C6" s="3" t="n">
-        <v>185</v>
-      </c>
-      <c r="D6" s="3" t="n">
         <v>0.01</v>
       </c>
     </row>

</xml_diff>